<commit_message>
Planilha de bancos de bateria atualizada automaticamente
</commit_message>
<xml_diff>
--- a/dados/Controle de Bancos de Bateria Oficial.xlsx
+++ b/dados/Controle de Bancos de Bateria Oficial.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\qinzen\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{0106F507-2DC0-43A4-BCD6-D174BEB4EC4F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="698" documentId="13_ncr:1_{AD74628D-BE06-4FC1-BE04-2187DD70E9AC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{EF93D86E-5E1A-41F8-A73E-47A300A18FE1}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="13905" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1825,7 +1825,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="28">
+  <cellXfs count="30">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -1884,6 +1884,10 @@
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" xr:uid="{00000000-000B-0000-0000-000008000000}"/>
@@ -2070,7 +2074,7 @@
       <numFmt numFmtId="30" formatCode="@"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="165" formatCode="dd/mm/yyyy"/>
+      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="30" formatCode="@"/>
@@ -2089,7 +2093,7 @@
       <numFmt numFmtId="30" formatCode="@"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="165" formatCode="dd/mm/yyyy"/>
+      <numFmt numFmtId="19" formatCode="dd/mm/yyyy"/>
       <alignment horizontal="left" vertical="center"/>
     </dxf>
     <dxf>
@@ -9005,56 +9009,56 @@
       <c r="M38" s="1"/>
       <c r="N38" s="1"/>
       <c r="O38" s="3"/>
-      <c r="P38" s="19"/>
+      <c r="P38" s="28"/>
       <c r="Q38" s="3"/>
       <c r="R38" s="3"/>
       <c r="S38" s="6"/>
       <c r="T38" s="3"/>
       <c r="U38" s="3"/>
       <c r="V38" s="3"/>
-      <c r="W38" s="12"/>
+      <c r="W38" s="29"/>
       <c r="X38" s="3"/>
       <c r="Y38" s="3"/>
       <c r="Z38" s="3"/>
       <c r="AA38" s="3"/>
       <c r="AB38" s="3"/>
       <c r="AC38" s="3"/>
-      <c r="AD38" s="12"/>
+      <c r="AD38" s="29"/>
       <c r="AE38" s="3"/>
       <c r="AF38" s="3"/>
       <c r="AG38" s="3"/>
       <c r="AH38" s="3"/>
       <c r="AI38" s="3"/>
       <c r="AJ38" s="3"/>
-      <c r="AK38" s="12"/>
+      <c r="AK38" s="29"/>
       <c r="AL38" s="3"/>
       <c r="AM38" s="3"/>
       <c r="AN38" s="3"/>
       <c r="AO38" s="3"/>
       <c r="AP38" s="3"/>
       <c r="AQ38" s="1"/>
-      <c r="AR38" s="12"/>
+      <c r="AR38" s="29"/>
       <c r="AS38" s="3"/>
       <c r="AT38" s="3"/>
       <c r="AU38" s="3"/>
       <c r="AV38" s="3"/>
       <c r="AW38" s="3"/>
       <c r="AX38" s="1"/>
-      <c r="AY38" s="12"/>
+      <c r="AY38" s="29"/>
       <c r="AZ38" s="3"/>
       <c r="BA38" s="3"/>
       <c r="BB38" s="3"/>
       <c r="BC38" s="3"/>
       <c r="BD38" s="3"/>
       <c r="BE38" s="1"/>
-      <c r="BF38" s="12"/>
+      <c r="BF38" s="29"/>
       <c r="BG38" s="3"/>
       <c r="BH38" s="3"/>
       <c r="BI38" s="3"/>
       <c r="BJ38" s="3"/>
       <c r="BK38" s="3"/>
       <c r="BL38" s="1"/>
-      <c r="BM38" s="12"/>
+      <c r="BM38" s="29"/>
       <c r="BN38" s="3"/>
       <c r="BO38" s="3"/>
       <c r="BP38" s="3"/>
@@ -9439,15 +9443,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x010100949757B2A3935B4A84A5374E630DBD2B" ma:contentTypeVersion="14" ma:contentTypeDescription="Crie um novo documento." ma:contentTypeScope="" ma:versionID="7a6d292a2f6a949c3af71fa212296ad8">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="337ea2d0-885f-4217-baff-63e0aa38c74f" xmlns:ns3="88b5053f-70bf-4e85-aff7-c22fa84ac4ca" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="20a9319f435276383e25e3a27c1527eb" ns2:_="" ns3:_="">
     <xsd:import namespace="337ea2d0-885f-4217-baff-63e0aa38c74f"/>
@@ -9674,6 +9669,15 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
@@ -9693,11 +9697,11 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{FC1EBE78-309B-4084-BAC4-28E69AD718B7}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{53916EA2-407A-40AC-B2E2-3247788E9B77}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{53916EA2-407A-40AC-B2E2-3247788E9B77}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{FC1EBE78-309B-4084-BAC4-28E69AD718B7}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>

</xml_diff>